<commit_message>
fixed excel file sheet name
</commit_message>
<xml_diff>
--- a/עדכון תוכנית שידורים TIAMO - שבועי.xlsx
+++ b/עדכון תוכנית שידורים TIAMO - שבועי.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RadioBot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{280F2FFC-9A88-4471-B3E2-6019BD53A9E2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5B117EC-2FAD-4F49-9820-C74C3405D236}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6280" xr2:uid="{582B9D01-2688-4D7A-A367-89A8B98C9EBD}"/>
   </bookViews>
   <sheets>
-    <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
+    <sheet name="תכנית חודשית" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -329,6 +329,23 @@
   </cellStyleXfs>
   <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -347,23 +364,6 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -682,622 +682,622 @@
   <dimension ref="A1:N14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.26953125" style="13" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="33.54296875" style="13" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.26953125" style="13" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="33.54296875" style="13" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.26953125" style="13" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="33.54296875" style="13" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.26953125" style="13" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="33.54296875" style="13" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.26953125" style="13" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="33.54296875" style="13" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.26953125" style="13" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="27.36328125" style="13" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.26953125" style="13" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="27.36328125" style="13" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="8.7265625" style="13"/>
+    <col min="1" max="1" width="11.26953125" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.54296875" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.26953125" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.54296875" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.26953125" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.54296875" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.26953125" style="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="33.54296875" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.26953125" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="33.54296875" style="5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.26953125" style="5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="27.36328125" style="5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.26953125" style="5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="27.36328125" style="5" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.7265625" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="2" t="s">
+      <c r="B1" s="7"/>
+      <c r="C1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="12"/>
-      <c r="E1" s="3" t="s">
+      <c r="D1" s="7"/>
+      <c r="E1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="12"/>
-      <c r="G1" s="4" t="s">
+      <c r="F1" s="7"/>
+      <c r="G1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="12"/>
-      <c r="I1" s="5" t="s">
+      <c r="H1" s="7"/>
+      <c r="I1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="12"/>
-      <c r="K1" s="6" t="s">
+      <c r="J1" s="7"/>
+      <c r="K1" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="12"/>
-      <c r="M1" s="7" t="s">
+      <c r="L1" s="7"/>
+      <c r="M1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="N1" s="12"/>
+      <c r="N1" s="7"/>
     </row>
     <row r="2" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="I2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="J2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="K2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="L2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="M2" s="8" t="s">
+      <c r="M2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="N2" s="8" t="s">
+      <c r="N2" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="I3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="J3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="K3" s="9" t="s">
+      <c r="K3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="L3" s="9" t="s">
+      <c r="L3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="M3" s="9" t="s">
+      <c r="M3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="N3" s="9" t="s">
+      <c r="N3" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="I4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="J4" s="9" t="s">
+      <c r="J4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="K4" s="9" t="s">
+      <c r="K4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="L4" s="9" t="s">
+      <c r="L4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M4" s="9" t="s">
+      <c r="M4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="N4" s="9" t="s">
+      <c r="N4" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I5" s="9" t="s">
+      <c r="I5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="J5" s="9" t="s">
+      <c r="J5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="K5" s="9" t="s">
+      <c r="K5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="L5" s="9" t="s">
+      <c r="L5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="M5" s="9" t="s">
+      <c r="M5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="N5" s="9" t="s">
+      <c r="N5" s="2" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I6" s="9" t="s">
+      <c r="I6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J6" s="9" t="s">
+      <c r="J6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="K6" s="9" t="s">
+      <c r="K6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="L6" s="9" t="s">
+      <c r="L6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="M6" s="9" t="s">
+      <c r="M6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="N6" s="9" t="s">
+      <c r="N6" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I7" s="9" t="s">
+      <c r="I7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J7" s="9" t="s">
+      <c r="J7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="K7" s="9" t="s">
+      <c r="K7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="L7" s="9" t="s">
+      <c r="L7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="M7" s="9" t="s">
+      <c r="M7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="N7" s="9" t="s">
+      <c r="N7" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="H8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="I8" s="9" t="s">
+      <c r="I8" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="J8" s="9" t="s">
+      <c r="J8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="K8" s="9" t="s">
+      <c r="K8" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L8" s="9" t="s">
+      <c r="L8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="M8" s="9" t="s">
+      <c r="M8" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="N8" s="9" t="s">
+      <c r="N8" s="2" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="H9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I9" s="9" t="s">
+      <c r="I9" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="J9" s="9" t="s">
+      <c r="J9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="K9" s="9" t="s">
+      <c r="K9" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="L9" s="9" t="s">
+      <c r="L9" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="M9" s="9" t="s">
+      <c r="M9" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="N9" s="9" t="s">
+      <c r="N9" s="2" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="H10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="I10" s="9" t="s">
+      <c r="I10" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="J10" s="9" t="s">
+      <c r="J10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="K10" s="9" t="s">
+      <c r="K10" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="L10" s="9" t="s">
+      <c r="L10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="M10" s="9" t="s">
+      <c r="M10" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="N10" s="9" t="s">
+      <c r="N10" s="2" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="H11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="I11" s="9" t="s">
+      <c r="I11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="J11" s="9" t="s">
+      <c r="J11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K11" s="9" t="s">
+      <c r="K11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="L11" s="9" t="s">
+      <c r="L11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="M11" s="9" t="s">
+      <c r="M11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="N11" s="9" t="s">
+      <c r="N11" s="2" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="D12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="F12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="H12" s="9" t="s">
+      <c r="H12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="I12" s="9" t="s">
+      <c r="I12" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="J12" s="9" t="s">
+      <c r="J12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="K12" s="9" t="s">
+      <c r="K12" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="L12" s="9" t="s">
+      <c r="L12" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="M12" s="9" t="s">
+      <c r="M12" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="N12" s="9" t="s">
+      <c r="N12" s="2" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="F13" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="H13" s="11" t="s">
+      <c r="H13" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="I13" s="9" t="s">
+      <c r="I13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="J13" s="11" t="s">
+      <c r="J13" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="K13" s="9" t="s">
+      <c r="K13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="L13" s="9" t="s">
+      <c r="L13" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="M13" s="9" t="s">
+      <c r="M13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="N13" s="9" t="s">
+      <c r="N13" s="2" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="E14" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="F14" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="G14" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="H14" s="9" t="s">
+      <c r="H14" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="I14" s="9" t="s">
+      <c r="I14" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="J14" s="9" t="s">
+      <c r="J14" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="K14" s="9" t="s">
+      <c r="K14" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="L14" s="9" t="s">
+      <c r="L14" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="M14" s="9" t="s">
+      <c r="M14" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="N14" s="9" t="s">
+      <c r="N14" s="2" t="s">
         <v>36</v>
       </c>
     </row>

</xml_diff>